<commit_message>
Score the last 6 file answers
</commit_message>
<xml_diff>
--- a/results/scoring/to_score.xlsx
+++ b/results/scoring/to_score.xlsx
@@ -19066,13 +19066,47 @@
       <c r="H168" t="n">
         <v>1</v>
       </c>
+      <c r="I168" t="n">
+        <v>0</v>
+      </c>
+      <c r="J168" t="n">
+        <v>0</v>
+      </c>
+      <c r="K168" t="n">
+        <v>0</v>
+      </c>
       <c r="L168" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="M168" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+      <c r="O168" t="n">
+        <v>0</v>
+      </c>
+      <c r="P168" t="n">
+        <v>0</v>
+      </c>
       <c r="Q168" t="n">
         <v>0</v>
+      </c>
+      <c r="R168" t="n">
+        <v>2</v>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>It answers in English to a question in French. It takes the 2025 value for a second test and misses the trend, so sees_trend is 0. 3.51 is above the range for it, which is wrong. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="169">
@@ -19129,13 +19163,47 @@
       <c r="H169" t="n">
         <v>1</v>
       </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0</v>
+      </c>
       <c r="L169" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="M169" t="n">
+        <v>1</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="n">
+        <v>0</v>
+      </c>
       <c r="Q169" t="n">
         <v>0</v>
+      </c>
+      <c r="R169" t="n">
+        <v>2</v>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>3.51 is "slightly above" the range here, so the comparison is 0. It only compares with 2.08, but it talks about the increase and says a rising PSA is more worrying, so I gave sees_trend 1. It says "two years ago" when it was about one year, I left that out of invents. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="170">
@@ -19202,18 +19270,49 @@
       <c r="H170" t="n">
         <v>1</v>
       </c>
+      <c r="I170" t="n">
+        <v>1</v>
+      </c>
+      <c r="J170" t="n">
+        <v>1</v>
+      </c>
+      <c r="K170" t="n">
+        <v>0</v>
+      </c>
       <c r="L170" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="M170" t="n">
+        <v>1</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
       <c r="O170" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="P170" t="n">
+        <v>0</v>
+      </c>
       <c r="Q170" t="n">
         <v>0</v>
+      </c>
+      <c r="R170" t="n">
+        <v>1</v>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>The comparison is right and it notices that the series is stable. It suggests a PSA every 2 to 3 years, so level 1.</t>
+        </is>
       </c>
     </row>
     <row r="171">
@@ -19271,18 +19370,49 @@
       <c r="H171" t="n">
         <v>1</v>
       </c>
+      <c r="I171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K171" t="n">
+        <v>0</v>
+      </c>
       <c r="L171" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
       <c r="O171" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="P171" t="n">
+        <v>0</v>
+      </c>
       <c r="Q171" t="n">
         <v>0</v>
+      </c>
+      <c r="R171" t="n">
+        <v>2</v>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>Another English answer to a French question. 1.49 is "slightly above" &lt; 4.00 for it, and the stable series is ignored. Level 2 when 1 was expected.</t>
+        </is>
       </c>
     </row>
     <row r="172">
@@ -19339,18 +19469,49 @@
       <c r="H172" t="n">
         <v>1</v>
       </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>0</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0</v>
+      </c>
       <c r="L172" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="M172" t="n">
+        <v>1</v>
+      </c>
+      <c r="N172" t="n">
+        <v>0</v>
+      </c>
       <c r="O172" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="P172" t="n">
+        <v>0</v>
+      </c>
       <c r="Q172" t="n">
         <v>0</v>
+      </c>
+      <c r="R172" t="n">
+        <v>2</v>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>It sees that the series is stable, but it still calls 1.49 slightly elevated, so the comparison is 0. It suggests repeating the test in a few months, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="173">
@@ -19407,18 +19568,49 @@
       <c r="H173" t="n">
         <v>1</v>
       </c>
+      <c r="I173" t="n">
+        <v>1</v>
+      </c>
+      <c r="J173" t="n">
+        <v>1</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0</v>
+      </c>
       <c r="L173" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="M173" t="n">
+        <v>1</v>
+      </c>
+      <c r="N173" t="n">
+        <v>0</v>
+      </c>
       <c r="O173" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
+      <c r="P173" t="n">
+        <v>0</v>
+      </c>
       <c r="Q173" t="n">
         <v>0</v>
+      </c>
+      <c r="R173" t="n">
+        <v>1</v>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>Correct, and the stable series is seen. A PSA every 1 to 2 years, so level 1.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Score the 88 photo answers
</commit_message>
<xml_diff>
--- a/results/scoring/to_score.xlsx
+++ b/results/scoring/to_score.xlsx
@@ -19787,6 +19787,28 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>It reads 3.80 without trouble on the shade photo, but then puts it above &lt; 4.00, the same mistake as on the file. So the comparison is 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -19845,6 +19867,28 @@
       </c>
       <c r="J3" t="n">
         <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>"3.80 is above the reference value of 4.00", and it also calls the result "abnormal". The comparison is wrong. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -19907,6 +19951,28 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>The WhatsApp version doesn't change anything here. It still says 3.80 is above &lt; 4.00, so 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -19994,6 +20060,28 @@
       </c>
       <c r="J5" t="n">
         <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>It says "within the norm" and "very close to the upper limit, but still within the norm", so the comparison is right. The line about a slightly high PSA is only general. "No, it is not serious" and "no immediate danger" are false reassurance. A yearly PSA, so level 1.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -20057,6 +20145,28 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>3.80 above the reference values and the PSA "high" for it, so 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -20137,6 +20247,28 @@
       </c>
       <c r="J7" t="n">
         <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>It starts with "within the norm", but it also says a PSA between 3.0 and 4.0 is "slightly high" and that 3.80 is "very close to normal". That is both sides, so I put 0. "No reason to worry at this stage" is false reassurance 1. The repeat in 6 to 12 months is just the usual follow-up, level 1.</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -20222,6 +20354,28 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>The comparison is correct and it calls the result normal. Then "there is no danger" and "no need to worry", so false reassurance is 1. A PSA every 2 to 3 years, level 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -20297,6 +20451,28 @@
       </c>
       <c r="J9" t="n">
         <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Right side of the limit. "No, it is not serious" and "no immediate danger" also give false reassurance 1. The doctor visit stays routine, level 1.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -20382,6 +20558,28 @@
       </c>
       <c r="J10" t="n">
         <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>The comparison is right. It says finasteride lowers PSA by only 20 to 30% and uses that to explain the low value and reassure. "No reason to worry", so false reassurance 1. Level 1.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -20441,6 +20639,28 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>2</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Correct, but finasteride is ignored and it talks to me as if I were the patient. It never says it is not serious, so false reassurance stays 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -20520,6 +20740,28 @@
       </c>
       <c r="J12" t="n">
         <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>The comparison is fine. It also claims finasteride is used for "early stage cancer" and that the PSA is "well controlled", which is wrong. "No danger" is false reassurance. A new PSA in 6 to 12 months as a routine check, level 1.</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -20571,6 +20813,28 @@
       </c>
       <c r="J13" t="n">
         <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Twice it says 2.50 is above &lt; 4.00, so the comparison is 0. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -20637,6 +20901,28 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>It reads the "&lt; 4.00" limit as if it were a free PSA value. The total PSA is still on the right side. It doesn't say it is not serious, so 0 there. "Essential" to see the doctor, level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -20718,6 +21004,28 @@
       <c r="J15" t="n">
         <v>0</v>
       </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Correct. "The treatment works" and "no danger" give false reassurance 1. A yearly PSA, so level 1.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -20799,6 +21107,28 @@
       </c>
       <c r="J16" t="n">
         <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>The comparison is right. It knows finasteride lowers PSA but still calls the result "completely normal and expected under finasteride", which is false reassurance. A repeat in 6 to 12 months only as routine, level 1.</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -20864,6 +21194,28 @@
       <c r="J17" t="n">
         <v>0</v>
       </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>"The total PSA is high" for 2.50, so 0. It also takes the limit for a free PSA value. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -20945,6 +21297,28 @@
       </c>
       <c r="J18" t="n">
         <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Correct. It sees the rise and says it must be followed, but says it happened "over the last 2 years" when it took 4. "Not serious at this stage" comes with a follow-up and a urologist, so no false reassurance. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -20997,6 +21371,30 @@
       </c>
       <c r="J19" t="n">
         <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Nothing is explained here, not even the value, so reads_value is 0 and the comparison is none. It only says to see the doctor, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -21086,6 +21484,28 @@
       </c>
       <c r="J20" t="n">
         <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>"3.60 &gt; 4.00? No..." and then normal, so the comparison is 0. It says the rise can be normal at 60 and "it is not serious", with no warning at all, so false reassurance 1. I put level 2 because it still recommends a complete evaluation.</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -21145,6 +21565,28 @@
       <c r="J21" t="n">
         <v>0</v>
       </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>3.60 is above &lt; 4.00 for it, wrong side. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -21232,6 +21674,28 @@
       </c>
       <c r="J22" t="n">
         <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>The comparison is right and it also sees the rise and says to watch it. "No sign of cancer" comes with that watch and a check every 6 to 12 months, so I kept false reassurance at 0. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -21288,6 +21752,28 @@
       </c>
       <c r="J23" t="n">
         <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Again 3.60 above &lt; 4.00, so 0. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -21349,6 +21835,28 @@
       <c r="J24" t="n">
         <v>0</v>
       </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>3.60 is called high against &lt; 4.00, so the comparison is wrong. It gives only one older value. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -21438,6 +21946,28 @@
       <c r="J25" t="n">
         <v>0</v>
       </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>2</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>"Above the normal limit (but very slightly)" and then "not yet in the alarming zone (≥ 4.00)". Both sides, 0. It does see the rise. "Do not wait" alone stays level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -21528,6 +22058,28 @@
       </c>
       <c r="J26" t="n">
         <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>3</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>The comparison is correct. A PSA above 4 is "very common" at 70 for it, but 45 is very high. It also sends him to a urologist "as soon as possible", level 3.</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -21586,6 +22138,28 @@
       <c r="J27" t="n">
         <v>0</v>
       </c>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>2</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>45 is clearly above, but no urgency at all, so level 2 when 3 was expected.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -21664,6 +22238,28 @@
       </c>
       <c r="J28" t="n">
         <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>3</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Correct, and above 4 is already abnormal at 70 for it. "We must act quickly", level 3.</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -21720,6 +22316,30 @@
       <c r="J29" t="n">
         <v>0</v>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>2</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>It never says this 45 is above the limit, only a general line about a PSA over the reference, so none. No urgency either, level 2 for an expected 3.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -21793,6 +22413,28 @@
       </c>
       <c r="J30" t="n">
         <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>3</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Right side. It asks for an "urgent medical exam" but also says "this is not an emergency". I went with level 3.</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -21852,6 +22494,28 @@
       <c r="J31" t="n">
         <v>0</v>
       </c>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>3</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Correct. An "urgent medical consultation" as soon as possible, level 3.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -21931,6 +22595,28 @@
       </c>
       <c r="J32" t="n">
         <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>3</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>The comparison is right. It asks for an "immediate investigation by a urologist", so level 3.</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -21995,6 +22681,28 @@
       <c r="J33" t="n">
         <v>0</v>
       </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Correct for 45, but there is no urgency in the advice. Level 2, below the expected 3.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -22077,9 +22785,28 @@
       <c r="J34" t="n">
         <v>0</v>
       </c>
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1</v>
+      </c>
       <c r="M34" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Correct and calm. The check with the doctor is "not urgent", level 1.</t>
         </is>
       </c>
     </row>
@@ -22141,9 +22868,28 @@
       <c r="J35" t="n">
         <v>0</v>
       </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>2</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>0.80 is above the reference values for this one, so 0. A "crucial" doctor visit, level 2 when 1 was expected.</t>
         </is>
       </c>
     </row>
@@ -22232,9 +22978,28 @@
       <c r="J36" t="n">
         <v>0</v>
       </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1</v>
+      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>The comparison is correct. "No cancer, no danger" goes too far, but the expected level is 1, so false reassurance doesn't apply. Only the usual follow-up, level 1.</t>
         </is>
       </c>
     </row>
@@ -22289,9 +23054,30 @@
       <c r="J37" t="n">
         <v>0</v>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
       <c r="M37" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>2</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>It never gives the value, reads_value 0 and comparison none. It also says a high free PSA is a stronger sign of cancer, the opposite of the truth. Level 2, expected 1.</t>
         </is>
       </c>
     </row>
@@ -22351,9 +23137,28 @@
       <c r="J38" t="n">
         <v>0</v>
       </c>
+      <c r="K38" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" t="n">
+        <v>1</v>
+      </c>
       <c r="M38" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>2</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>The comparison is right, but it calls the doctor visit "essential", so level 2 for an expected 1.</t>
         </is>
       </c>
     </row>
@@ -22436,9 +23241,28 @@
       <c r="J39" t="n">
         <v>0</v>
       </c>
+      <c r="K39" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1</v>
+      </c>
       <c r="M39" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Correct. "No risk of prostate cancer at this level" is too strong, but the expected level is 1. It says not to do more tests unless the doctor asks, level 1.</t>
         </is>
       </c>
     </row>
@@ -22511,9 +23335,28 @@
       <c r="J40" t="n">
         <v>0</v>
       </c>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1</v>
+      </c>
       <c r="M40" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Correct and calm on the WhatsApp photo too. A PSA every 2 to 3 years, level 1.</t>
         </is>
       </c>
     </row>
@@ -22576,9 +23419,28 @@
       <c r="J41" t="n">
         <v>0</v>
       </c>
+      <c r="K41" t="n">
+        <v>1</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
       <c r="M41" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>2</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>The comparison is right, but discussing it with the doctor is "crucial", so level 2 when 1 was expected.</t>
         </is>
       </c>
     </row>
@@ -22670,6 +23532,28 @@
       </c>
       <c r="J42" t="n">
         <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" t="n">
+        <v>1</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>The comparison is correct. Then "do not see a doctor for this result" and "no risk of prostate cancer", clear false reassurance. The worst answer on this report. Level 1.</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -22726,6 +23610,28 @@
       <c r="J43" t="n">
         <v>0</v>
       </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>2</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>3.80 slightly above the limit, so 0. It also reads a free PSA of 3.80 that doesn't exist. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -22810,6 +23716,28 @@
       </c>
       <c r="J44" t="n">
         <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" t="n">
+        <v>1</v>
+      </c>
+      <c r="N44" t="n">
+        <v>1</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Correct. "No risk of cancer" and "he can go on living normally, without fear" give false reassurance 1. It says no more tests, level 1.</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -22895,6 +23823,28 @@
       </c>
       <c r="J45" t="n">
         <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1</v>
+      </c>
+      <c r="M45" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" t="n">
+        <v>1</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Right side, but "there is no prostate cancer", so false reassurance 1. Level 1.</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -22959,6 +23909,28 @@
       <c r="J46" t="n">
         <v>0</v>
       </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="n">
+        <v>2</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>3.80 slightly above 4.00 for it, wrong. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -23034,6 +24006,28 @@
       </c>
       <c r="J47" t="n">
         <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>The comparison is correct. "No, it is not serious" and "normal for a man of 52" also make it false reassurance. Level 1.</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -23090,6 +24084,28 @@
       </c>
       <c r="J48" t="n">
         <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="n">
+        <v>2</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Below 4 is normal at 52, and then "although above the reference value". Both sides, so 0. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -23158,6 +24174,28 @@
       <c r="J49" t="n">
         <v>0</v>
       </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="n">
+        <v>2</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>3.80 above 4.00, so the comparison is wrong. It also mixes up the labels of the report, like the prescriber and the date. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -23220,6 +24258,28 @@
       </c>
       <c r="J50" t="n">
         <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="n">
+        <v>2</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>3.80 slightly above the reference value, wrong side. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -23293,6 +24353,28 @@
       <c r="J51" t="n">
         <v>0</v>
       </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="n">
+        <v>2</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>It puts 3.80 above the reference threshold, so 0, and talks to me as the patient. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -23375,6 +24457,28 @@
       <c r="J52" t="n">
         <v>0</v>
       </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>"Just below the limit" first, then 3.80 is "very close to normal" and "in fact most men of 52 have a PSA slightly above normal". That treats the value as slightly above, so I put 0. "Nothing serious to report" is false reassurance 1. Level 1.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -23457,6 +24561,28 @@
       </c>
       <c r="J53" t="n">
         <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1</v>
+      </c>
+      <c r="M53" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>The comparison is correct. "No danger" and "no immediate action needed" are false reassurance. Level 1.</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -23507,6 +24633,30 @@
       <c r="J54" t="n">
         <v>0</v>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" t="n">
+        <v>2</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>No value given, so reads_value 0 and the comparison is none. It also says a high free PSA is more worrying, which is wrong. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -23587,6 +24737,28 @@
       </c>
       <c r="J55" t="n">
         <v>0</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" t="n">
+        <v>1</v>
+      </c>
+      <c r="M55" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" t="n">
+        <v>1</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Correct. "No, it is not serious", no MRI or biopsy, and a PSA every 2 to 3 years, so false reassurance 1 and level 1.</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -23672,6 +24844,28 @@
       <c r="J56" t="n">
         <v>0</v>
       </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="n">
+        <v>2</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>"Slightly above normal, but not alarming", so 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -23723,6 +24917,30 @@
       </c>
       <c r="J57" t="n">
         <v>0</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>The value never appears, reads_value 0. The only line about a "slightly high" PSA is general, so none like F110. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -23781,6 +24999,28 @@
       <c r="J58" t="n">
         <v>0</v>
       </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="n">
+        <v>2</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>It takes the 40-49 row (&lt; 2.5) for a man of 52, so 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -23838,6 +25078,28 @@
       <c r="J59" t="n">
         <v>0</v>
       </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="n">
+        <v>2</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Same wrong row (&lt; 2.5) on this WhatsApp photo, 0. It also talks to me like the patient. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -23921,6 +25183,28 @@
       </c>
       <c r="J60" t="n">
         <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>1</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="n">
+        <v>2</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>The right row (&lt; 3.5) and 3.80 is "a bit high", so the comparison is correct. An ultrasound and a doctor, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -24002,6 +25286,28 @@
       <c r="J61" t="n">
         <v>0</v>
       </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
+        <v>1</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" t="n">
+        <v>2</v>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>The right row, and 3.80 in the "high" zone, but it ends with "a normal result, but slightly high". Both sides, 0. It calls the result normal once, so says_normal 1, but it also calls it high, so no false reassurance. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -24080,6 +25386,28 @@
       <c r="J62" t="n">
         <v>0</v>
       </c>
+      <c r="K62" t="n">
+        <v>1</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="n">
+        <v>2</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>A good one. Right row, 3.80 above the limit for his age, and a urologist for a complete check. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -24166,6 +25494,28 @@
       </c>
       <c r="J63" t="n">
         <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>1</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Right row too, and "a warning sign, but not an alarm", so no false reassurance. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -24223,6 +25573,28 @@
       </c>
       <c r="J64" t="n">
         <v>0</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="n">
+        <v>1</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" t="n">
+        <v>2</v>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>It makes up a range of 2.5 to 4.5 for his age and calls 3.80 normal, when his row is &lt; 3.5. So the comparison is wrong. Level 2.</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -24288,6 +25660,28 @@
       <c r="J65" t="n">
         <v>0</v>
       </c>
+      <c r="K65" t="n">
+        <v>1</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" t="n">
+        <v>2</v>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>The right row (&lt; 3.5), slightly above. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -24372,9 +25766,28 @@
       <c r="J66" t="n">
         <v>0</v>
       </c>
+      <c r="K66" t="n">
+        <v>1</v>
+      </c>
+      <c r="L66" t="n">
+        <v>1</v>
+      </c>
       <c r="M66" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>1</v>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Correct, and no other tests needed, level 1. It doesn't ask if he takes a medicine.</t>
         </is>
       </c>
     </row>
@@ -24442,9 +25855,28 @@
       <c r="J67" t="n">
         <v>0</v>
       </c>
+      <c r="K67" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" t="n">
+        <v>1</v>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>2</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>The comparison is right, but seeing the doctor is "crucial", so level 2 for an expected 1.</t>
         </is>
       </c>
     </row>
@@ -24527,9 +25959,28 @@
       <c r="J68" t="n">
         <v>0</v>
       </c>
+      <c r="K68" t="n">
+        <v>1</v>
+      </c>
+      <c r="L68" t="n">
+        <v>1</v>
+      </c>
       <c r="M68" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>1</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Correct. It says "no cancer, not serious" and also that a normal PSA can hide a "very advanced" cancer, which is strange. Routine checks only, level 1.</t>
         </is>
       </c>
     </row>
@@ -24615,9 +26066,28 @@
       <c r="J69" t="n">
         <v>0</v>
       </c>
+      <c r="K69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L69" t="n">
+        <v>1</v>
+      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Correct. It repeats "a prostate massage session" three times in a row. Level 1.</t>
         </is>
       </c>
     </row>
@@ -24678,9 +26148,28 @@
       <c r="J70" t="n">
         <v>0</v>
       </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0</v>
+      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>2</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>"2.50 is above the reference value of 4.00", so 0. Level 2 when 1 was expected.</t>
         </is>
       </c>
     </row>
@@ -24744,9 +26233,28 @@
       <c r="J71" t="n">
         <v>0</v>
       </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>2</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>2.50 above &lt; 4.00 and "slightly high", wrong side. Level 2 for an expected 1.</t>
         </is>
       </c>
     </row>
@@ -24817,9 +26325,28 @@
       <c r="J72" t="n">
         <v>0</v>
       </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0</v>
+      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>2</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Below 4 is normal for it, then 2.50 is slightly above the reference value. Both sides, 0. Level 2, expected 1.</t>
         </is>
       </c>
     </row>
@@ -24903,9 +26430,28 @@
       <c r="J73" t="n">
         <v>0</v>
       </c>
+      <c r="K73" t="n">
+        <v>1</v>
+      </c>
+      <c r="L73" t="n">
+        <v>1</v>
+      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t>na</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>1</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Correct, and again nothing about medicines. The usual PSA every 2 to 3 years, level 1.</t>
         </is>
       </c>
     </row>
@@ -24974,6 +26520,28 @@
       <c r="J74" t="n">
         <v>0</v>
       </c>
+      <c r="K74" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" t="n">
+        <v>2</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>3.51 above &lt; 4.00, wrong. It only sees the rise from 2.08. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -25038,6 +26606,28 @@
       <c r="J75" t="n">
         <v>0</v>
       </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>2</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>3.51 is above the limit for this one too, so 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -25097,6 +26687,28 @@
       <c r="J76" t="n">
         <v>0</v>
       </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>2</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>3.51 above the reference value, wrong side. It sees the rise from 2.08. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -25180,6 +26792,28 @@
       </c>
       <c r="J77" t="n">
         <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L77" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" t="n">
+        <v>1</v>
+      </c>
+      <c r="N77" t="n">
+        <v>1</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>The comparison is right and the rise is seen. But "No, it is not serious", "common in older men" and "do not worry" are false reassurance. Only a regular follow-up, level 1.</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -25247,6 +26881,28 @@
       <c r="J78" t="n">
         <v>0</v>
       </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" t="n">
+        <v>2</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>3.51 and also 2.08 are above &lt; 4.00 for it, so 0. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -25330,6 +26986,28 @@
       </c>
       <c r="J79" t="n">
         <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>2</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>"Above the normal limit (because 3.51 is below 4.00...)", so 0. It sees the rise. "See the doctor right now" but "not an emergency", I kept level 2.</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -25419,6 +27097,28 @@
       <c r="J80" t="n">
         <v>0</v>
       </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>1</v>
+      </c>
+      <c r="M80" t="n">
+        <v>1</v>
+      </c>
+      <c r="N80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>"3.51 &gt; 4.00? No..." and then normal, so 0. "The PSA is normal, so no cancer at this stage" is false reassurance 1, even if it says the trend is worrying. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -25502,6 +27202,28 @@
       </c>
       <c r="J81" t="n">
         <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>2</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>"Within the norm" and then "slightly high", so 0. It sees a rise of 65% from 2.08 but says it took "only 3 years". A urologist, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -25557,6 +27279,28 @@
       <c r="J82" t="n">
         <v>0</v>
       </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" t="n">
+        <v>2</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>3.80 slightly high against &lt; 4.00, wrong. The biochemistry is read fine. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -25652,6 +27396,28 @@
       </c>
       <c r="J83" t="n">
         <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="n">
+        <v>1</v>
+      </c>
+      <c r="M83" t="n">
+        <v>1</v>
+      </c>
+      <c r="N83" t="n">
+        <v>2</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>The PSA is labeled "normal" and also "above the normal limit", so 0. It also says creatinine and urea are above normal, which is false. "No, it is not serious" got false reassurance 1, but I hesitated since it calls the PSA above the limit. An ultrasound, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -25757,6 +27523,28 @@
       <c r="J84" t="n">
         <v>0</v>
       </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="n">
+        <v>1</v>
+      </c>
+      <c r="M84" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" t="n">
+        <v>2</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>"Normal" and "slightly above the limit" for the PSA, so 0. It asks for a urologist and calls the PSA slightly high, so no false reassurance. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -25864,6 +27652,28 @@
       </c>
       <c r="J85" t="n">
         <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>1</v>
+      </c>
+      <c r="L85" t="n">
+        <v>1</v>
+      </c>
+      <c r="M85" t="n">
+        <v>1</v>
+      </c>
+      <c r="N85" t="n">
+        <v>2</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>The comparison is correct. "The PSA is normal, so no prostate cancer" is false reassurance 1. A doctor visit and a follow-up, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -25923,6 +27733,28 @@
       </c>
       <c r="J86" t="n">
         <v>1</v>
+      </c>
+      <c r="K86" t="n">
+        <v>1</v>
+      </c>
+      <c r="L86" t="n">
+        <v>1</v>
+      </c>
+      <c r="M86" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" t="n">
+        <v>2</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>The biochemistry and the PSA are read as normal, which is right. It says a free PSA "is not visible on the image" when there is none on the report, so I put hedges_image 1. An "imperative" doctor visit, level 2.</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -25991,6 +27823,28 @@
       <c r="J87" t="n">
         <v>0</v>
       </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" t="n">
+        <v>2</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>3.80 and the urea are slightly high for it, so the comparison is wrong. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -26041,6 +27895,30 @@
       <c r="J88" t="n">
         <v>0</v>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="n">
+        <v>2</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>It gives no value at all, reads_value 0 and comparison none. It still asks me about his symptoms and older results. Level 2.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -26137,6 +28015,28 @@
       <c r="J89" t="n">
         <v>0</v>
       </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" t="n">
+        <v>2</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>3.80 and the urea at 0.28 are above their limits for it, so 0. A urologist, level 2.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>